<commit_message>
feat: KS-2 +Код ВОР, KS-6 4-section rewrite, +5 VOR prices
</commit_message>
<xml_diff>
--- a/report/templates/ВОР_с_расценками.xlsx
+++ b/report/templates/ВОР_с_расценками.xlsx
@@ -1128,7 +1128,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:HL853"/>
+  <dimension ref="A1:HL858"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.109375" defaultRowHeight="13.8"/>
   <cols>
     <col width="9.109375" customWidth="1" style="136" min="1" max="1"/>
@@ -62618,6 +62618,186 @@
       <c r="HK853" s="16" t="n"/>
       <c r="HL853" s="16" t="n"/>
     </row>
+    <row r="854">
+      <c r="A854" s="33" t="inlineStr">
+        <is>
+          <t>3 этап</t>
+        </is>
+      </c>
+      <c r="B854" s="34" t="inlineStr">
+        <is>
+          <t>3.3.2</t>
+        </is>
+      </c>
+      <c r="C854" s="35" t="inlineStr">
+        <is>
+          <t>Устройство монолитного железобетонного перекрытия здания Общежития</t>
+        </is>
+      </c>
+      <c r="D854" s="36" t="inlineStr">
+        <is>
+          <t>м3</t>
+        </is>
+      </c>
+      <c r="E854" s="144" t="n">
+        <v>208.6</v>
+      </c>
+      <c r="F854" s="145" t="n">
+        <v>80000</v>
+      </c>
+      <c r="G854" s="145" t="n">
+        <v>16688000</v>
+      </c>
+      <c r="H854" s="10" t="inlineStr">
+        <is>
+          <t>По аналогу 3.2.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" s="33" t="inlineStr">
+        <is>
+          <t>3 этап</t>
+        </is>
+      </c>
+      <c r="B855" s="34" t="inlineStr">
+        <is>
+          <t>3.3.2.1</t>
+        </is>
+      </c>
+      <c r="C855" s="35" t="inlineStr">
+        <is>
+          <t>Армирование плиты перекрытия арматурой ø8А500С, отм. +6,590</t>
+        </is>
+      </c>
+      <c r="D855" s="36" t="inlineStr">
+        <is>
+          <t>кг</t>
+        </is>
+      </c>
+      <c r="E855" s="144" t="n">
+        <v>7981.29</v>
+      </c>
+      <c r="F855" s="145" t="n">
+        <v>100</v>
+      </c>
+      <c r="G855" s="145" t="n">
+        <v>798129</v>
+      </c>
+      <c r="H855" s="10" t="inlineStr">
+        <is>
+          <t>Экспертная оценка</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" s="33" t="inlineStr">
+        <is>
+          <t>3 этап</t>
+        </is>
+      </c>
+      <c r="B856" s="34" t="inlineStr">
+        <is>
+          <t>3.3.2.2</t>
+        </is>
+      </c>
+      <c r="C856" s="35" t="inlineStr">
+        <is>
+          <t>Армирование плиты перекрытия арматурой ø8А500С, отм. +9,930</t>
+        </is>
+      </c>
+      <c r="D856" s="36" t="inlineStr">
+        <is>
+          <t>кг</t>
+        </is>
+      </c>
+      <c r="E856" s="144" t="n">
+        <v>7982.29</v>
+      </c>
+      <c r="F856" s="145" t="n">
+        <v>100</v>
+      </c>
+      <c r="G856" s="145" t="n">
+        <v>798229</v>
+      </c>
+      <c r="H856" s="10" t="inlineStr">
+        <is>
+          <t>Экспертная оценка</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" s="33" t="inlineStr">
+        <is>
+          <t>3 этап</t>
+        </is>
+      </c>
+      <c r="B857" s="34" t="inlineStr">
+        <is>
+          <t>3.3.6</t>
+        </is>
+      </c>
+      <c r="C857" s="35" t="inlineStr">
+        <is>
+          <t>Устройство монолитного железобетонного перекрытия переходной Галереи</t>
+        </is>
+      </c>
+      <c r="D857" s="36" t="inlineStr">
+        <is>
+          <t>м3</t>
+        </is>
+      </c>
+      <c r="E857" s="144" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="F857" s="145" t="n">
+        <v>80000</v>
+      </c>
+      <c r="G857" s="145" t="n">
+        <v>224000</v>
+      </c>
+      <c r="H857" s="10" t="inlineStr">
+        <is>
+          <t>По аналогу 3.2.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" s="33" t="inlineStr">
+        <is>
+          <t>7 этап</t>
+        </is>
+      </c>
+      <c r="B858" s="34" t="inlineStr">
+        <is>
+          <t>7.2.1.1</t>
+        </is>
+      </c>
+      <c r="C858" s="35" t="inlineStr">
+        <is>
+          <t>Разработка грунта</t>
+        </is>
+      </c>
+      <c r="D858" s="36" t="inlineStr">
+        <is>
+          <t>м3</t>
+        </is>
+      </c>
+      <c r="E858" s="144" t="n">
+        <v>887.7</v>
+      </c>
+      <c r="F858" s="145" t="n">
+        <v>11800</v>
+      </c>
+      <c r="G858" s="145" t="n">
+        <v>10474860</v>
+      </c>
+      <c r="H858" s="10" t="inlineStr">
+        <is>
+          <t>По аналогичным земляным работам</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="8" scale="38" fitToHeight="0"/>

</xml_diff>